<commit_message>
결과 파일 업데이트 2026-09-20 10:36
</commit_message>
<xml_diff>
--- a/results/andar_할인율모니터링_20260920.xlsx
+++ b/results/andar_할인율모니터링_20260920.xlsx
@@ -571,12 +571,12 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
@@ -613,7 +613,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>3,590</t>
+          <t>3,593</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -655,7 +655,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>3,590</t>
+          <t>3,593</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1213,84 +1213,84 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=5845&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13862&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>EJFMT-01</t>
+          <t>EOTBG-03</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>릴렉스 에어소프트 요가매트 (8mm)</t>
+          <t>데이 앤 트래블 숄더백</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>31,000</t>
+          <t>79,000</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>31,000</t>
+          <t>59,000</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>25%</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>10,109</t>
+          <t>127</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13862&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=5845&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>EOTBG-03</t>
+          <t>EJFMT-01</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>데이 앤 트래블 숄더백</t>
+          <t>릴렉스 에어소프트 요가매트 (8mm)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>79,000</t>
+          <t>31,000</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>59,000</t>
+          <t>31,000</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>127</t>
+          <t>10,110</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
@@ -1411,7 +1411,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>141</t>
+          <t>142</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1453,7 +1453,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>8,168</t>
+          <t>8,171</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1537,7 +1537,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>426</t>
+          <t>428</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -1579,7 +1579,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>426</t>
+          <t>428</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -1621,7 +1621,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>426</t>
+          <t>428</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -1675,84 +1675,84 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13409&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=12318&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>EOTBG-10</t>
+          <t>ENTBG-13</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>에어플라이 투웨이 프리런 백 3.0</t>
+          <t>데일리 스퀘어백</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>35,000</t>
+          <t>69,000</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>35,000</t>
+          <t>49,000</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>29%</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>1,151</t>
+          <t>434</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=12318&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13409&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>ENTBG-13</t>
+          <t>EOTBG-10</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>데일리 스퀘어백</t>
+          <t>에어플라이 투웨이 프리런 백 3.0</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>69,000</t>
+          <t>35,000</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>49,000</t>
+          <t>35,000</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>29%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>434</t>
+          <t>1,151</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>3.0</t>
         </is>
       </c>
     </row>
@@ -1789,7 +1789,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>1,416</t>
+          <t>1,417</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -1843,84 +1843,84 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15372&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13215&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>EOTBG-16</t>
+          <t>EOTCP-01</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>폴더블 미니백 2.0</t>
+          <t>올라운드 버킷햇</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>39,000</t>
+          <t>69,000</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>29,000</t>
+          <t>69,000</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>26%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>297</t>
+          <t>367</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13215&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15372&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>EOTCP-01</t>
+          <t>EOTBG-16</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>올라운드 버킷햇</t>
+          <t>폴더블 미니백 2.0</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>69,000</t>
+          <t>39,000</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>69,000</t>
+          <t>29,000</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>26%</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>364</t>
+          <t>297</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
@@ -2011,27 +2011,27 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=14059&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13838&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>ENTSO-02</t>
+          <t>EOTFB-01</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>안다르 제트플라이 (우먼즈)</t>
+          <t>에어쿨링 와이드 헤드밴드</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>139,000</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>139,000</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2041,7 +2041,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>1,044</t>
+          <t>2,454</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -2058,7 +2058,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>ENTSO-12</t>
+          <t>ENTSO-02</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2083,7 +2083,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>1,044</t>
+          <t>1,045</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -2095,27 +2095,27 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13838&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=14059&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>EOTFB-01</t>
+          <t>ENTSO-12</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>에어쿨링 와이드 헤드밴드</t>
+          <t>안다르 제트플라이 (우먼즈)</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>139,000</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>139,000</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2125,7 +2125,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>2,452</t>
+          <t>1,045</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -2209,7 +2209,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>57</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -2347,37 +2347,37 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15143&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8819&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>EOTBG-17</t>
+          <t>EMTSC-04</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>3 in 1 캐리온 더플백</t>
+          <t>[1&amp;1] 논슬립 서포트 하프 토삭스 (HOLE &amp; SOLID)</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>109,000</t>
+          <t>19,800</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>85,000</t>
+          <t>15,800</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>22%</t>
+          <t>20%</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>3,217</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -2394,7 +2394,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>EMTSC-04</t>
+          <t>EMTSC-05</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2419,7 +2419,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>3,216</t>
+          <t>3,217</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -2431,37 +2431,37 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8819&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15143&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>EMTSC-05</t>
+          <t>EOTBG-17</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>[1&amp;1] 논슬립 서포트 하프 토삭스 (HOLE &amp; SOLID)</t>
+          <t>3 in 1 캐리온 더플백</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>19,800</t>
+          <t>109,000</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>15,800</t>
+          <t>85,000</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>20%</t>
+          <t>22%</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>3,216</t>
+          <t>46</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -2515,27 +2515,27 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16031&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15629&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>EOTGL-02</t>
+          <t>EOTBG-23</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>히트 런 글러브</t>
+          <t>안다르 실버 리유저블백 M</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>29,000</t>
+          <t>6,500</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>29,000</t>
+          <t>6,500</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -2545,7 +2545,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>386</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -2599,42 +2599,42 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15629&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15153&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>EOTBG-23</t>
+          <t>EOTSC-13</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>안다르 실버 리유저블백 M</t>
+          <t>테이핑 러닝 삭스</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>6,500</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>6,500</t>
+          <t>7,900</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>43%</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>385</t>
+          <t>283</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
@@ -2725,27 +2725,27 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=17425&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13853&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>EPTSC-06</t>
+          <t>EOTBG-12</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>필라테스 크루 삭스</t>
+          <t>프리런 벨크로 러닝 벨트</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>35,000</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>35,000</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -2755,7 +2755,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>92</t>
+          <t>248</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -2767,27 +2767,27 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13853&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=17425&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>EOTBG-12</t>
+          <t>EPTSC-06</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>프리런 벨크로 러닝 벨트</t>
+          <t>필라테스 크루 삭스</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>35,000</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>35,000</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -2797,7 +2797,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>248</t>
+          <t>92</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -2809,69 +2809,69 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15153&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=10940&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>EOTSC-13</t>
+          <t>ENTBG-03</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>테이핑 러닝 삭스</t>
+          <t>데일리 스트링 쇼퍼백</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>79,000</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>7,900</t>
+          <t>79,000</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>43%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>282</t>
+          <t>738</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=10940&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13843&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>ENTBG-03</t>
+          <t>EOTBG-02</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>데일리 스트링 쇼퍼백</t>
+          <t>액티브 라이트 백팩</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>79,000</t>
+          <t>69,000</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>79,000</t>
+          <t>69,000</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -2881,39 +2881,39 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>736</t>
+          <t>383</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13843&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16031&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>EOTBG-02</t>
+          <t>EOTGL-02</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>액티브 라이트 백팩</t>
+          <t>히트 런 글러브</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>69,000</t>
+          <t>29,000</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>69,000</t>
+          <t>29,000</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -2923,7 +2923,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>382</t>
+          <t>220</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -3007,7 +3007,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>301</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
@@ -3061,42 +3061,42 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=5145&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13604&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>EJPFR-04</t>
+          <t>EOTSV-01</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>릴렉스 폼롤러 Ⅱ</t>
+          <t>[1&amp;1] 하이 서포트 무릎 보호대</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>39,000</t>
+          <t>29,800</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>39,000</t>
+          <t>24,900</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>16%</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>6,369</t>
+          <t>716</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
@@ -3145,79 +3145,79 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13859&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16660&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>ENTSO-12</t>
+          <t>EOTET-03</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>안다르 제트플라이 (맨즈)</t>
+          <t>맨즈 라이트 러닝 베스트</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>139,000</t>
+          <t>79,000</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>139,000</t>
+          <t>55,000</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>30%</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>696</t>
+          <t>12</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.6</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13604&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=9996&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>EOTSV-01</t>
+          <t>EMTSC-27</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>[1&amp;1] 하이 서포트 무릎 보호대</t>
+          <t>올라운드 오버 니삭스</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>29,800</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>24,900</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>16%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>714</t>
+          <t>297</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -3229,69 +3229,69 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16660&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=17423&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>EOTET-03</t>
+          <t>EPTSC-04</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>맨즈 라이트 러닝 베스트</t>
+          <t>필라테스 토삭스</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>79,000</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>55,000</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>105</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=17423&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13859&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>EPTSC-04</t>
+          <t>ENTSO-12</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>필라테스 토삭스</t>
+          <t>안다르 제트플라이 (맨즈)</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>139,000</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>139,000</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -3301,39 +3301,39 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>105</t>
+          <t>696</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=9996&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=17437&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>EMTSC-27</t>
+          <t>EPTCP-03</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>올라운드 오버 니삭스</t>
+          <t>썬가드 와이드 버킷햇</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>69,000</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>69,000</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -3343,29 +3343,29 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>297</t>
+          <t>68</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.6</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13410&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16631&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>EOTSC-09</t>
+          <t>EPTSV-03</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>컴프레션 러닝 니삭스</t>
+          <t>컴프레션 카프 슬리브 (종아리 보호대)</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -3385,39 +3385,39 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>353</t>
+          <t>255</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=17437&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13410&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>EPTCP-03</t>
+          <t>EOTSC-09</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>썬가드 와이드 버킷햇</t>
+          <t>컴프레션 러닝 니삭스</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>69,000</t>
+          <t>14,900</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>69,000</t>
+          <t>14,900</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -3427,39 +3427,39 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>353</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16631&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=10948&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>EPTSV-03</t>
+          <t>ENTSC-20</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>컴프레션 카프 슬리브 (종아리 보호대)</t>
+          <t>시그니처 로고 크루 삭스</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>14,900</t>
+          <t>7,900</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>14,900</t>
+          <t>7,900</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -3469,7 +3469,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>590</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
@@ -3481,27 +3481,27 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=11962&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13854&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>ENTMT-01</t>
+          <t>EOTSC-06</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>레스트 인 마블 요가매트 (4mm)</t>
+          <t>서포트 쿠션 러닝 삭스</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>49,000</t>
+          <t>10,900</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>49,000</t>
+          <t>10,900</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -3511,7 +3511,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>770</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
@@ -3523,27 +3523,27 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=6660&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=11962&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>EKPMT-03</t>
+          <t>ENTMT-01</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>릴렉스 논슬립 요가 타월</t>
+          <t>레스트 인 마블 요가매트 (4mm)</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>35,900</t>
+          <t>49,000</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>35,900</t>
+          <t>49,000</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -3553,49 +3553,49 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>1,564</t>
+          <t>270</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15385&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=6660&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>EOTSC-16</t>
+          <t>EKPMT-03</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>[1&amp;1] 논슬립 스킨 토삭스</t>
+          <t>릴렉스 논슬립 요가 타월</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>25,800</t>
+          <t>35,900</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>19,900</t>
+          <t>35,900</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>23%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>528</t>
+          <t>1,564</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
@@ -3612,7 +3612,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>EOTSC-17</t>
+          <t>EOTSC-16</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -3649,37 +3649,37 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=10948&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15385&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>ENTSC-20</t>
+          <t>EOTSC-17</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>시그니처 로고 크루 삭스</t>
+          <t>[1&amp;1] 논슬립 스킨 토삭스</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>7,900</t>
+          <t>25,800</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>7,900</t>
+          <t>19,900</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>23%</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>590</t>
+          <t>528</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
@@ -3691,27 +3691,27 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13854&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=5837&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>EOTSC-06</t>
+          <t>EJFMB-03</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>서포트 쿠션 러닝 삭스</t>
+          <t>릴렉스 짐볼 65cm</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>10,900</t>
+          <t>19,000</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>10,900</t>
+          <t>19,000</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -3721,39 +3721,39 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>770</t>
+          <t>2,119</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=5837&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16847&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>EJFMB-03</t>
+          <t>EPTSC-02</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>릴렉스 짐볼 65cm</t>
+          <t>하이 쿠션 테이핑 러닝 삭스</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>19,000</t>
+          <t>12,900</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>19,000</t>
+          <t>12,900</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -3763,54 +3763,54 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>2,119</t>
+          <t>101</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16847&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=10953&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>EPTSC-02</t>
+          <t>ENTSC-07</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>하이 쿠션 테이핑 러닝 삭스</t>
+          <t>[3 SET] 에어컴피 크루 삭스</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>12,900</t>
+          <t>51,000</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>12,900</t>
+          <t>29,000</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>43%</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>101</t>
+          <t>562</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
@@ -3847,7 +3847,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>640</t>
+          <t>641</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -3859,27 +3859,27 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=10554&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16637&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>ENTMK-01</t>
+          <t>EPTFB-02</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>UV 프로텍션 맨즈 골프 마스크</t>
+          <t>퍼포먼스 심리스 손목밴드</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>23,000</t>
+          <t>6,900</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>23,000</t>
+          <t>6,900</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -3889,7 +3889,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>1,539</t>
+          <t>286</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
@@ -3901,37 +3901,37 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=11130&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13405&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>ENTSV-01</t>
+          <t>EOTSV-01</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>[1&amp;1] 3D 쿨링 팔토시</t>
+          <t>하이 서포트 무릎 보호대</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>29,800</t>
+          <t>14,900</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>25,900</t>
+          <t>14,900</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>13%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>558</t>
+          <t>716</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
@@ -3943,84 +3943,84 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=10953&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=10554&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>ENTSC-07</t>
+          <t>ENTMK-01</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>[3 SET] 에어컴피 크루 삭스</t>
+          <t>UV 프로텍션 맨즈 골프 마스크</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>51,000</t>
+          <t>23,000</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>29,000</t>
+          <t>23,000</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>43%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>562</t>
+          <t>1,539</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16637&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15431&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>EPTFB-02</t>
+          <t>ENTSC-19</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>퍼포먼스 심리스 손목밴드</t>
+          <t>[1&amp;1] 맨즈 논슬립 토삭스</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>6,900</t>
+          <t>23,800</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>6,900</t>
+          <t>16,900</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>29%</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>285</t>
+          <t>315</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
@@ -4032,7 +4032,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>ENTSC-19</t>
+          <t>EOTSC-14</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -4069,37 +4069,37 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15431&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8769&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>EOTSC-14</t>
+          <t>EMTSV-02</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>[1&amp;1] 맨즈 논슬립 토삭스</t>
+          <t>서포트 발목 보호대</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>23,800</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>16,900</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>29%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>315</t>
+          <t>727</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
@@ -4111,69 +4111,69 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16650&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=11130&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>EPTCP-02</t>
+          <t>ENTSV-01</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>시그니처 로고 나일론 볼캡</t>
+          <t>[1&amp;1] 3D 쿨링 팔토시</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>39,000</t>
+          <t>29,800</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>39,000</t>
+          <t>25,900</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>13%</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>558</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8769&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16650&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>EMTSV-02</t>
+          <t>EPTCP-02</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>서포트 발목 보호대</t>
+          <t>시그니처 로고 나일론 볼캡</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>39,000</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>39,000</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -4183,39 +4183,39 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>727</t>
+          <t>69</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13851&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=11459&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>EOTCP-03</t>
+          <t>ENTSC-14</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>쿨 라운드 볼캡</t>
+          <t>논슬립 퍼포먼스 니삭스</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>45,000</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>45,000</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -4225,7 +4225,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>107</t>
+          <t>753</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
@@ -4237,27 +4237,27 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=11459&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8578&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>ENTSC-14</t>
+          <t>EMTSC-01</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>논슬립 퍼포먼스 니삭스</t>
+          <t>링글 크루 삭스</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>7,900</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>7,900</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
@@ -4267,7 +4267,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>753</t>
+          <t>1,335</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
@@ -4279,27 +4279,27 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=11458&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13407&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>ENTSC-13</t>
+          <t>EOTSV-03</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>논슬립 퍼포먼스 크루삭스</t>
+          <t>서포트 허리 보호대</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>11,900</t>
+          <t>34,000</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>11,900</t>
+          <t>34,000</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
@@ -4309,7 +4309,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>668</t>
+          <t>186</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
@@ -4321,27 +4321,27 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13405&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8728&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>EOTSV-01</t>
+          <t>EMTSC-05</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>하이 서포트 무릎 보호대</t>
+          <t>논슬립 서포트 하프 토삭스 (SOLID)</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>14,900</t>
+          <t>9,900</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>14,900</t>
+          <t>9,900</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
@@ -4351,39 +4351,39 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>714</t>
+          <t>569</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8578&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=11458&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>EMTSC-01</t>
+          <t>ENTSC-13</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>링글 크루 삭스</t>
+          <t>논슬립 퍼포먼스 크루삭스</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>7,900</t>
+          <t>11,900</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>7,900</t>
+          <t>11,900</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -4393,12 +4393,12 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>1,335</t>
+          <t>668</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
@@ -4435,7 +4435,7 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>1,376</t>
+          <t>1,377</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
@@ -4477,7 +4477,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>1,376</t>
+          <t>1,377</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
@@ -4519,7 +4519,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>1,376</t>
+          <t>1,377</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
@@ -4531,27 +4531,27 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13407&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=6661&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>EOTSV-03</t>
+          <t>EKPMB-01</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>서포트 허리 보호대</t>
+          <t>릴렉스 웨이트볼 0.5kg</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>34,000</t>
+          <t>6,900</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>34,000</t>
+          <t>6,900</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
@@ -4561,7 +4561,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>699</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
@@ -4573,37 +4573,37 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8728&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=10657&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>EMTSC-05</t>
+          <t>EMTSC-17</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>논슬립 서포트 하프 토삭스 (SOLID)</t>
+          <t>[3 SET] 맨즈 클래식 삭스</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>9,900</t>
+          <t>20,700</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>9,900</t>
+          <t>17,900</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>14%</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>569</t>
+          <t>230</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
@@ -4657,27 +4657,27 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=6661&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=12480&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>EKPMB-01</t>
+          <t>ENTSC-24</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>릴렉스 웨이트볼 0.5kg</t>
+          <t>웜 슬릿 레그 워머</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>6,900</t>
+          <t>29,000</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>6,900</t>
+          <t>29,000</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -4687,39 +4687,39 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>699</t>
+          <t>297</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.6</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=12480&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8621&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>ENTSC-24</t>
+          <t>EMTSV-06</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>웜 슬릿 레그 워머</t>
+          <t>에어쿨링 손목 보호대</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>29,000</t>
+          <t>15,900</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>29,000</t>
+          <t>15,900</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -4729,49 +4729,49 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>297</t>
+          <t>1,101</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=10657&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13404&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>EMTSC-17</t>
+          <t>EOTGL-01</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>[3 SET] 맨즈 클래식 삭스</t>
+          <t>짐 글러브 2.0</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>20,700</t>
+          <t>25,000</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>17,900</t>
+          <t>25,000</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>14%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>230</t>
+          <t>292</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
@@ -4783,27 +4783,27 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8621&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=17424&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>EMTSV-06</t>
+          <t>EPTSC-05</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>에어쿨링 손목 보호대</t>
+          <t>필라테스 앵클 삭스</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>15,900</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>15,900</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -4813,39 +4813,39 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>1,101</t>
+          <t>42</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13404&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16045&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>EOTGL-01</t>
+          <t>EOTMU-01</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>짐 글러브 2.0</t>
+          <t>스트링 패딩 넥워머</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>25,000</t>
+          <t>49,000</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>25,000</t>
+          <t>49,000</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
@@ -4855,91 +4855,91 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>292</t>
+          <t>46</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8837&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=11039&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>EMTSV-02</t>
+          <t>ENTFB-01</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>[1&amp;1] 서포트 발목 보호대</t>
+          <t>에어쿨링 라인 스크런치</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>27,800</t>
+          <t>8,900</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>22,900</t>
+          <t>8,900</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>727</t>
+          <t>777</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=6664&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8837&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>EKPRB-04</t>
+          <t>EMTSV-02</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>릴렉스 3레벨 스트레칭 롱밴드</t>
+          <t>[1&amp;1] 서포트 발목 보호대</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>34,900</t>
+          <t>27,800</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>34,900</t>
+          <t>22,900</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>18%</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>470</t>
+          <t>727</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
@@ -4993,27 +4993,27 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=17424&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=6664&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>EPTSC-05</t>
+          <t>EKPRB-04</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>필라테스 앵클 삭스</t>
+          <t>릴렉스 3레벨 스트레칭 롱밴드</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>34,900</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>34,900</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
@@ -5023,39 +5023,39 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>470</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16045&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=6662&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>EOTMU-01</t>
+          <t>EKPMB-02</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>스트링 패딩 넥워머</t>
+          <t>릴렉스 미니 짐볼</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>49,000</t>
+          <t>13,000</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>49,000</t>
+          <t>13,000</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
@@ -5065,12 +5065,12 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>1,235</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.6</t>
         </is>
       </c>
     </row>
@@ -5119,79 +5119,79 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=6662&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=10191&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>EKPMB-02</t>
+          <t>EMTSC-26</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>릴렉스 미니 짐볼</t>
+          <t>[1&amp;1] 램스울 크루 삭스</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>13,000</t>
+          <t>19,800</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>13,000</t>
+          <t>17,900</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>10%</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>1,235</t>
+          <t>850</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=10191&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=5145&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>EMTSC-26</t>
+          <t>EJPFR-04</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>[1&amp;1] 램스울 크루 삭스</t>
+          <t>릴렉스 폼롤러 Ⅱ</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>19,800</t>
+          <t>39,000</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>17,900</t>
+          <t>39,000</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>10%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>847</t>
+          <t>6,370</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
@@ -5233,7 +5233,7 @@
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>354</t>
+          <t>355</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
@@ -5371,27 +5371,27 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15734&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15377&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>EOTSC-20</t>
+          <t>EOTGL-04</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>레그 미들 워머</t>
+          <t>논슬립 스킨 요기 글러브</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>12,900</t>
+          <t>10,900</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>12,900</t>
+          <t>10,900</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
@@ -5401,39 +5401,39 @@
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>199</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.5</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15377&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15734&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>EOTGL-04</t>
+          <t>EOTSC-20</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>논슬립 스킨 요기 글러브</t>
+          <t>레그 미들 워머</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>10,900</t>
+          <t>12,900</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>10,900</t>
+          <t>12,900</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -5443,39 +5443,39 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>199</t>
+          <t>38</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13805&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=12793&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>EOTSC-04</t>
+          <t>ENTMU-01</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>올데이 수피마 스니커즈 삭스</t>
+          <t>소프트 니트 머플러</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>5,900</t>
+          <t>19,900</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>5,900</t>
+          <t>19,900</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -5485,7 +5485,7 @@
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>434</t>
+          <t>472</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
@@ -5497,27 +5497,27 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=12793&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=6665&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>ENTMU-01</t>
+          <t>EKPRB-05</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>소프트 니트 머플러</t>
+          <t>릴렉스 4레벨 힙 밴드</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>19,900</t>
+          <t>21,900</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>19,900</t>
+          <t>21,900</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
@@ -5527,7 +5527,7 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>472</t>
+          <t>527</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
@@ -5539,27 +5539,27 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=6665&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=12096&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>EKPRB-05</t>
+          <t>ENTET-02</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>릴렉스 4레벨 힙 밴드</t>
+          <t>릴렉스 소프트 웨이트바 2kg</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>21,900</t>
+          <t>39,000</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>21,900</t>
+          <t>39,000</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
@@ -5569,12 +5569,12 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>527</t>
+          <t>76</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
@@ -5611,7 +5611,7 @@
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>594</t>
+          <t>595</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
@@ -5623,27 +5623,27 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16034&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15733&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>EOTGL-03</t>
+          <t>EOTSC-19</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>소프트 니트 플립 글러브</t>
+          <t>레그 숏 워머</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>23,900</t>
+          <t>10,900</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>23,900</t>
+          <t>10,900</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
@@ -5653,7 +5653,7 @@
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>86</t>
+          <t>14</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
@@ -5665,27 +5665,27 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15733&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13805&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>EOTSC-19</t>
+          <t>EOTSC-04</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>레그 숏 워머</t>
+          <t>올데이 수피마 스니커즈 삭스</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>10,900</t>
+          <t>5,900</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>10,900</t>
+          <t>5,900</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
@@ -5695,7 +5695,7 @@
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>435</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
@@ -5791,37 +5791,37 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=11039&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15719&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>ENTFB-01</t>
+          <t>EOTSC-19</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>에어쿨링 라인 스크런치</t>
+          <t>[1&amp;1] 레그 워머</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>8,900</t>
+          <t>21,800</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>8,900</t>
+          <t>15,900</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>27%</t>
         </is>
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>776</t>
+          <t>234</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
@@ -5833,79 +5833,79 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=12096&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15719&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>ENTET-02</t>
+          <t>EOTSC-20</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>릴렉스 소프트 웨이트바 2kg</t>
+          <t>[1&amp;1] 레그 워머</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>39,000</t>
+          <t>21,800</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>39,000</t>
+          <t>15,900</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>27%</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>234</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15719&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13566&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>EOTSC-19</t>
+          <t>EOTSC-10</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>[1&amp;1] 레그 워머</t>
+          <t>시그니처 로고 맨즈 크루 삭스</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>21,800</t>
+          <t>7,900</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>15,900</t>
+          <t>7,900</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>27%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>233</t>
+          <t>219</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
@@ -5917,42 +5917,42 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15719&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16034&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>EOTSC-20</t>
+          <t>EOTGL-03</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>[1&amp;1] 레그 워머</t>
+          <t>소프트 니트 플립 글러브</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>21,800</t>
+          <t>23,900</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>15,900</t>
+          <t>23,900</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>27%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>233</t>
+          <t>86</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
@@ -6031,7 +6031,7 @@
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>624</t>
+          <t>625</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
@@ -6085,27 +6085,27 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13566&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=14562&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>EOTSC-10</t>
+          <t>EOTBG-11</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>시그니처 로고 맨즈 크루 삭스</t>
+          <t>메쉬 파우치</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>7,900</t>
+          <t>29,000</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>7,900</t>
+          <t>29,000</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
@@ -6115,39 +6115,39 @@
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>219</t>
+          <t>195</t>
         </is>
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=14562&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=14561&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>EOTBG-11</t>
+          <t>EOTBG-05</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>메쉬 파우치</t>
+          <t>메쉬 포켓 비치백</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>29,000</t>
+          <t>49,000</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>29,000</t>
+          <t>49,000</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
@@ -6157,39 +6157,39 @@
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>194</t>
+          <t>63</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13806&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=14085&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>EOTSC-05</t>
+          <t>EOTSV-04</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>올데이 수피마 앵클 삭스</t>
+          <t>프리런 라이트 러닝 밴드</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>6,900</t>
+          <t>32,000</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>6,900</t>
+          <t>32,000</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
@@ -6199,39 +6199,39 @@
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>479</t>
+          <t>129</t>
         </is>
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.2</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=14561&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=11457&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>EOTBG-05</t>
+          <t>ENTSC-12</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>메쉬 포켓 비치백</t>
+          <t>논슬립 퍼포먼스 토삭스</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>49,000</t>
+          <t>12,900</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>49,000</t>
+          <t>12,900</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
@@ -6241,39 +6241,39 @@
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>63</t>
+          <t>4,136</t>
         </is>
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=14085&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13851&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>EOTSV-04</t>
+          <t>EOTCP-03</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>프리런 라이트 러닝 밴드</t>
+          <t>쿨 라운드 볼캡</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>32,000</t>
+          <t>45,000</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>32,000</t>
+          <t>45,000</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
@@ -6283,39 +6283,39 @@
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>129</t>
+          <t>107</t>
         </is>
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>4.2</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=11457&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=12795&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>ENTSC-12</t>
+          <t>ENTCP-05</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>논슬립 퍼포먼스 토삭스</t>
+          <t>소프트 니트 비니</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>12,900</t>
+          <t>19,900</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>12,900</t>
+          <t>19,900</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
@@ -6325,7 +6325,7 @@
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>4,136</t>
+          <t>364</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
@@ -6337,27 +6337,27 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=12795&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16035&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>ENTCP-05</t>
+          <t>EOTSC-12</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>소프트 니트 비니</t>
+          <t>소프트 니트 기모 니삭스</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>19,900</t>
+          <t>15,900</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>19,900</t>
+          <t>15,900</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
@@ -6367,39 +6367,39 @@
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>364</t>
+          <t>102</t>
         </is>
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>5.0</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16035&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=9993&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>EOTSC-12</t>
+          <t>EMTSC-29</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>소프트 니트 기모 니삭스</t>
+          <t>니트 루즈 삭스</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>15,900</t>
+          <t>9,900</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>15,900</t>
+          <t>9,900</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
@@ -6409,39 +6409,39 @@
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>102</t>
+          <t>513</t>
         </is>
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=9993&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=12488&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>EMTSC-29</t>
+          <t>ENTBG-10</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>니트 루즈 삭스</t>
+          <t>스퀘어 크로스백</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>9,900</t>
+          <t>79,000</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>9,900</t>
+          <t>79,000</t>
         </is>
       </c>
       <c r="F144" t="inlineStr">
@@ -6451,7 +6451,7 @@
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>513</t>
+          <t>634</t>
         </is>
       </c>
       <c r="H144" t="inlineStr">
@@ -6463,27 +6463,27 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=12488&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=17386&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>ENTBG-10</t>
+          <t>EPTSC-07</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>스퀘어 크로스백</t>
+          <t>맨즈 필라테스 앵클 삭스</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>79,000</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>79,000</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="F145" t="inlineStr">
@@ -6493,29 +6493,29 @@
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>634</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>5.0</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=17386&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8770&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>EPTSC-07</t>
+          <t>EMTSV-03</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>맨즈 필라테스 앵클 삭스</t>
+          <t>서포트 무릎 보호대</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -6535,39 +6535,39 @@
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>2,027</t>
         </is>
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>4.5</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8770&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13806&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>EMTSV-03</t>
+          <t>EOTSC-05</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>서포트 무릎 보호대</t>
+          <t>올데이 수피마 앵클 삭스</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>6,900</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>6,900</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
@@ -6577,12 +6577,12 @@
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>2,027</t>
+          <t>480</t>
         </is>
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
@@ -6631,69 +6631,69 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=11061&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13605&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>ENTSV-01</t>
+          <t>EOTSV-02</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>3D 쿨링 팔토시</t>
+          <t>[1&amp;1] 하이 서포트 팔꿈치 보호대</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>14,900</t>
+          <t>29,800</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>14,900</t>
+          <t>24,900</t>
         </is>
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>16%</t>
         </is>
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>558</t>
+          <t>156</t>
         </is>
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13842&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=11061&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>EOTBG-04</t>
+          <t>ENTSV-01</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>데님 포켓 숄더백</t>
+          <t>3D 쿨링 팔토시</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>59,000</t>
+          <t>14,900</t>
         </is>
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>59,000</t>
+          <t>14,900</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
@@ -6703,39 +6703,39 @@
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>558</t>
         </is>
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=9988&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13842&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>EMTSC-26</t>
+          <t>EOTBG-04</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>램스울 크루 삭스</t>
+          <t>데님 포켓 숄더백</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>9,900</t>
+          <t>59,000</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>9,900</t>
+          <t>59,000</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
@@ -6745,7 +6745,7 @@
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>340</t>
+          <t>39</t>
         </is>
       </c>
       <c r="H151" t="inlineStr">
@@ -6757,27 +6757,27 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=17842&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15732&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>EPTSC-03</t>
+          <t>EOTSC-11</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>데일리 루즈 삭스</t>
+          <t>웜 레그 롱 워머</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>11,900</t>
+          <t>25,000</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>11,900</t>
+          <t>25,000</t>
         </is>
       </c>
       <c r="F152" t="inlineStr">
@@ -6787,7 +6787,7 @@
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>113</t>
         </is>
       </c>
       <c r="H152" t="inlineStr">
@@ -6799,27 +6799,27 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8727&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=9988&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>EMTSC-04</t>
+          <t>EMTSC-26</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>논슬립 서포트 하프 토삭스 (HOLE)</t>
+          <t>램스울 크루 삭스</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>10,900</t>
+          <t>9,900</t>
         </is>
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>10,900</t>
+          <t>9,900</t>
         </is>
       </c>
       <c r="F153" t="inlineStr">
@@ -6829,7 +6829,7 @@
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>646</t>
+          <t>342</t>
         </is>
       </c>
       <c r="H153" t="inlineStr">
@@ -6841,27 +6841,27 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8768&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=17842&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>EMTSV-01</t>
+          <t>EPTSC-03</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>서포트 팔꿈치 보호대</t>
+          <t>데일리 루즈 삭스</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>11,900</t>
         </is>
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>11,900</t>
         </is>
       </c>
       <c r="F154" t="inlineStr">
@@ -6871,39 +6871,39 @@
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>594</t>
+          <t>29</t>
         </is>
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=11963&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8727&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>ENTSC-19</t>
+          <t>EMTSC-04</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>맨즈 논슬립 하프 토삭스</t>
+          <t>논슬립 서포트 하프 토삭스 (HOLE)</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>11,900</t>
+          <t>10,900</t>
         </is>
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>11,900</t>
+          <t>10,900</t>
         </is>
       </c>
       <c r="F155" t="inlineStr">
@@ -6913,39 +6913,39 @@
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>94</t>
+          <t>646</t>
         </is>
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=12778&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8768&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>ENTBG-14</t>
+          <t>EMTSV-01</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>웨이브 패딩 파우치</t>
+          <t>서포트 팔꿈치 보호대</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>32,000</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>32,000</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
@@ -6955,81 +6955,81 @@
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>195</t>
+          <t>595</t>
         </is>
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13605&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=11963&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>EOTSV-02</t>
+          <t>ENTSC-19</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>[1&amp;1] 하이 서포트 팔꿈치 보호대</t>
+          <t>맨즈 논슬립 하프 토삭스</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>29,800</t>
+          <t>11,900</t>
         </is>
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>24,900</t>
+          <t>11,900</t>
         </is>
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>16%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>156</t>
+          <t>94</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13406&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=12778&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>EOTSV-02</t>
+          <t>ENTBG-14</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>하이 서포트 팔꿈치 보호대</t>
+          <t>웨이브 패딩 파우치</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>14,900</t>
+          <t>32,000</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>14,900</t>
+          <t>32,000</t>
         </is>
       </c>
       <c r="F158" t="inlineStr">
@@ -7039,7 +7039,7 @@
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>156</t>
+          <t>195</t>
         </is>
       </c>
       <c r="H158" t="inlineStr">
@@ -7051,27 +7051,27 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15732&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13406&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>EOTSC-11</t>
+          <t>EOTSV-02</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>웜 레그 롱 워머</t>
+          <t>하이 서포트 팔꿈치 보호대</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>25,000</t>
+          <t>14,900</t>
         </is>
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>25,000</t>
+          <t>14,900</t>
         </is>
       </c>
       <c r="F159" t="inlineStr">
@@ -7081,7 +7081,7 @@
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>113</t>
+          <t>156</t>
         </is>
       </c>
       <c r="H159" t="inlineStr">
@@ -7585,7 +7585,7 @@
       </c>
       <c r="G171" t="inlineStr">
         <is>
-          <t>373</t>
+          <t>374</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">

</xml_diff>